<commit_message>
Updated the qualitative evaluation for case 1 and case 2
</commit_message>
<xml_diff>
--- a/evaluation/results/Qualitative-Evaluation-Case1.xlsx
+++ b/evaluation/results/Qualitative-Evaluation-Case1.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DSouzaJ\Datasets\subject-indexing-dataset\evaluation\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SadruddinS\Data\GermEval25\Code\subject-indexing-dataset\evaluation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D125A174-1FB9-48B9-A277-93323F771269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="6" r:id="rId1"/>
@@ -114,7 +113,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
@@ -361,7 +360,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.39E-2</c:v>
+                  <c:v>0.47870000000000001</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0.76739999999999997</c:v>
@@ -513,7 +512,7 @@
                   <c:v>0.74609999999999999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.51200000000000001</c:v>
+                  <c:v>0.51329999999999998</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.77029999999999998</c:v>
@@ -531,7 +530,7 @@
                   <c:v>0.95220000000000005</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>9.0399999999999994E-2</c:v>
+                  <c:v>0.46079999999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0.66569999999999996</c:v>
@@ -683,7 +682,7 @@
                   <c:v>0.7762</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.56220000000000003</c:v>
+                  <c:v>0.57050000000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.77029999999999998</c:v>
@@ -701,7 +700,7 @@
                   <c:v>0.91669999999999996</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2344</c:v>
+                  <c:v>0.5353</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0.66569999999999996</c:v>
@@ -853,7 +852,7 @@
                   <c:v>0.82799999999999996</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.64</c:v>
+                  <c:v>0.64870000000000005</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.77029999999999998</c:v>
@@ -871,7 +870,7 @@
                   <c:v>0.96109999999999995</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.38769999999999999</c:v>
+                  <c:v>0.6038</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0.66569999999999996</c:v>
@@ -942,7 +941,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="de-DE"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="860198751"/>
@@ -1001,7 +1000,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="de-DE"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="860198271"/>
@@ -1018,6 +1017,7 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
+      <c:layout/>
       <c:overlay val="1"/>
       <c:spPr>
         <a:noFill/>
@@ -1043,7 +1043,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -1073,7 +1073,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="de-DE"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1952,7 +1952,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2152,52 +2152,52 @@
         <v>18</v>
       </c>
       <c r="C4" s="2">
-        <v>0.36399999999999999</v>
+        <v>0.44800000000000001</v>
       </c>
       <c r="D4" s="2">
-        <v>0.24149999999999999</v>
+        <v>0.29499999999999998</v>
       </c>
       <c r="E4" s="2">
-        <v>0.43059999999999998</v>
+        <v>0.51949999999999996</v>
       </c>
       <c r="F4" s="2">
-        <v>0.29039999999999999</v>
+        <v>0.35570000000000002</v>
       </c>
       <c r="G4" s="2">
-        <v>0.32</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="H4" s="2">
-        <v>0.37659999999999999</v>
+        <v>0.43869999999999998</v>
       </c>
       <c r="I4" s="2">
-        <v>0.42749999999999999</v>
+        <v>0.50180000000000002</v>
       </c>
       <c r="J4" s="2">
-        <v>0.34599999999999997</v>
+        <v>0.39910000000000001</v>
       </c>
       <c r="K4" s="2">
-        <v>0.32129999999999997</v>
+        <v>0.33600000000000002</v>
       </c>
       <c r="L4" s="2">
-        <v>0.5877</v>
+        <v>0.6331</v>
       </c>
       <c r="M4" s="2">
-        <v>0.49419999999999997</v>
+        <v>0.55600000000000005</v>
       </c>
       <c r="N4" s="2">
-        <v>0.41549999999999998</v>
+        <v>0.439</v>
       </c>
       <c r="O4" s="2">
         <v>0.31900000000000001</v>
       </c>
       <c r="P4" s="2">
-        <v>0.75449999999999995</v>
+        <v>0.75719999999999998</v>
       </c>
       <c r="Q4" s="3">
-        <v>0.57509999999999994</v>
+        <v>0.62</v>
       </c>
       <c r="R4" s="2">
-        <v>0.44840000000000002</v>
+        <v>0.44890000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -2207,7 +2207,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2448,7 +2448,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2689,7 +2689,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2879,49 +2879,49 @@
         <v>0.46</v>
       </c>
       <c r="C4" s="2">
-        <v>0.30520000000000003</v>
+        <v>0.30830000000000002</v>
       </c>
       <c r="D4" s="2">
         <v>0.53779999999999994</v>
       </c>
       <c r="E4" s="2">
-        <v>0.3669</v>
+        <v>0.36919999999999997</v>
       </c>
       <c r="F4" s="2">
         <v>0.4</v>
       </c>
       <c r="G4" s="2">
-        <v>0.44109999999999999</v>
+        <v>0.44829999999999998</v>
       </c>
       <c r="H4" s="2">
-        <v>0.51200000000000001</v>
+        <v>0.51329999999999998</v>
       </c>
       <c r="I4" s="2">
-        <v>0.41949999999999998</v>
+        <v>0.42280000000000001</v>
       </c>
       <c r="J4" s="2">
         <v>0.39329999999999998</v>
       </c>
       <c r="K4" s="2">
-        <v>0.66080000000000005</v>
+        <v>0.67330000000000001</v>
       </c>
       <c r="L4" s="2">
-        <v>0.56220000000000003</v>
+        <v>0.57050000000000001</v>
       </c>
       <c r="M4" s="2">
-        <v>0.49309999999999998</v>
+        <v>0.4965</v>
       </c>
       <c r="N4" s="2">
         <v>0.36499999999999999</v>
       </c>
       <c r="O4" s="2">
-        <v>0.82509999999999994</v>
+        <v>0.83850000000000002</v>
       </c>
       <c r="P4" s="3">
-        <v>0.64</v>
+        <v>0.64870000000000005</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.50609999999999999</v>
+        <v>0.50860000000000005</v>
       </c>
     </row>
   </sheetData>
@@ -2930,7 +2930,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3171,7 +3171,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3358,40 +3358,40 @@
         <v>18</v>
       </c>
       <c r="B4" s="2">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="C4" s="2">
-        <v>0.01</v>
+        <v>0.2747</v>
       </c>
       <c r="D4" s="2">
-        <v>3.39E-2</v>
+        <v>0.47870000000000001</v>
       </c>
       <c r="E4" s="2">
-        <v>0</v>
+        <v>0.3322</v>
       </c>
       <c r="F4" s="2">
-        <v>0.1</v>
+        <v>0.33</v>
       </c>
       <c r="G4" s="2">
-        <v>0.1023</v>
+        <v>0.40560000000000002</v>
       </c>
       <c r="H4" s="2">
-        <v>9.0399999999999994E-2</v>
+        <v>0.46079999999999999</v>
       </c>
       <c r="I4" s="2">
-        <v>0.1011</v>
+        <v>0.3639</v>
       </c>
       <c r="J4" s="2">
-        <v>0.24</v>
+        <v>0.31330000000000002</v>
       </c>
       <c r="K4" s="2">
-        <v>0.36220000000000002</v>
+        <v>0.57689999999999997</v>
       </c>
       <c r="L4" s="2">
-        <v>0.2344</v>
+        <v>0.5353</v>
       </c>
       <c r="M4" s="2">
-        <v>0.28870000000000001</v>
+        <v>0.40610000000000002</v>
       </c>
       <c r="N4" s="2">
         <v>0.31</v>
@@ -3400,7 +3400,7 @@
         <v>0.70760000000000001</v>
       </c>
       <c r="P4" s="3">
-        <v>0.38769999999999999</v>
+        <v>0.6038</v>
       </c>
       <c r="Q4" s="2">
         <v>0.43109999999999998</v>
@@ -3412,7 +3412,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9A76718-CDA5-4B72-9506-40FAB67B475B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B5:G24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3583,13 +3583,13 @@
         <v>0.53779999999999994</v>
       </c>
       <c r="E14" s="2">
-        <v>0.51200000000000001</v>
+        <v>0.51329999999999998</v>
       </c>
       <c r="F14" s="2">
-        <v>0.56220000000000003</v>
+        <v>0.57050000000000001</v>
       </c>
       <c r="G14" s="3">
-        <v>0.64</v>
+        <v>0.64870000000000005</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
@@ -3718,16 +3718,16 @@
         <v>18</v>
       </c>
       <c r="D22" s="2">
-        <v>3.39E-2</v>
+        <v>0.47870000000000001</v>
       </c>
       <c r="E22" s="2">
-        <v>9.0399999999999994E-2</v>
+        <v>0.46079999999999999</v>
       </c>
       <c r="F22" s="2">
-        <v>0.2344</v>
+        <v>0.5353</v>
       </c>
       <c r="G22" s="3">
-        <v>0.38769999999999999</v>
+        <v>0.6038</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">

</xml_diff>